<commit_message>
added Sharon Welch to advisor info list
Email sharon@sizemoreinsurance.com inferred from existing firstname@sizemoreinsurance.com naming convention — please confirm.
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="600" yWindow="600" windowWidth="37800" windowHeight="20040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="1" max="1"/>
@@ -1231,8 +1231,6 @@
           <t>john@sizemoreinsurance.com</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1250,8 +1248,6 @@
           <t>jj@sizemoreinsurance.com</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1277,6 +1273,33 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>910-444-0923</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Oleander</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sharon Welch</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>sharon@sizemoreinsurance.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>4815 Oleander Dr, STE 101 Wilmington, NC 28403</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>910-208-6452</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added Elizabeth Hullender to advisor info list
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="1" max="1"/>
@@ -1303,6 +1303,33 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Shallotte</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Elizabeth Hullender</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>elizabeth@sizemoreinsurance.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>4702 Main Street Shallotte, NC 28470</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>910-383-9946</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added Kate Carson to advisor info list
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="600" yWindow="600" windowWidth="37800" windowHeight="20040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="1" max="1"/>
@@ -1330,6 +1330,33 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Oleander</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Kate Carson</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>kate@sizemoreinsurance.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>4815 Oleander Dr, STE 101 Wilmington, NC 28403</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>910-791-1011</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Marissa Schultz, Sharon Jordan, Troy Anderson and Amber Kirkpatrick from advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R32648fb8ee094919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R4fb48ead94c344eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,31 +655,11 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oleander</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Troy Anderson</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">troy@sizemoreinsurance.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4815 Oleander Dr, STE 101 Wilmington, NC 28403</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">910-791-1011</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="inlineStr">
@@ -763,31 +743,11 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shallotte</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Amber Kirkpatrick</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">amber@sizemoreinsurance.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4702 Main Street Shallotte, NC 28470</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">910-754-4366</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="inlineStr">
@@ -817,31 +777,11 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shallotte</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Marissa Schultz</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">marissa@sizemoreinsurance.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4702 Main Street Shallotte, NC 28470</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">910-754-4366</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="inlineStr">
@@ -952,31 +892,11 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hampstead</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sharon Jordan</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sharonj@sizemoreinsurance.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16406 Hwy Ste 6, Hampstead, NC 28433</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">910-270-9111</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Add Debi Benson to Shallotte Snapshot advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R4fb48ead94c344eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R272322341a4849ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1142,6 +1142,23 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>Shallotte</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Debi Benson</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>debi@sizemoreinsurance.com</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>4702 Main Street Shallotte, NC 28470</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>910-754-4366</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Luke Gullicksen to Oleander Snapshot advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -1159,6 +1159,23 @@
         <x:v>910-754-4366</x:v>
       </x:c>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>Oleander</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Luke Gullicksen</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>Luke@sizemoreinsurance.com</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>4815 Oleander Dr, STE 101 Wilmington, NC 28403</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>910-791-1011</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Correct Luke Gullickson display name in Snapshot advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R272322341a4849ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R6ddeff59e1344a90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1164,7 +1164,7 @@
         <x:v>Oleander</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>Luke Gullicksen</x:v>
+        <x:v>Luke Gullickson</x:v>
       </x:c>
       <x:c r="C36" t="str">
         <x:v>Luke@sizemoreinsurance.com</x:v>

</xml_diff>

<commit_message>
Add Charles Neely (Shallotte) to Snapshot advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -1176,6 +1176,23 @@
         <x:v>910-791-1011</x:v>
       </x:c>
     </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>Shallotte</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Charles Neely</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>charles@sizemoreinsurance.com</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>4702 Main Street Shallotte, NC 28470</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>910-754-4366</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Jason Carter (Oleander) to Snapshot advisor roster
</commit_message>
<xml_diff>
--- a/backend/advisor_info_list/advisor_info_list.xlsx
+++ b/backend/advisor_info_list/advisor_info_list.xlsx
@@ -1193,6 +1193,23 @@
         <x:v>910-754-4366</x:v>
       </x:c>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>Oleander</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Jason Carter</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>jason@sizemoreinsurance.com</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>4815 Oleander Dr, STE 101 Wilmington, NC 28403</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>910-791-1011</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>